<commit_message>
enhance projects ui and update marn photos
</commit_message>
<xml_diff>
--- a/data/projects.xlsx
+++ b/data/projects.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Makled\Desktop\portfolio, cv\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D55B2C47-B3A5-4906-80D4-A211FD1AE128}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B6ED814-5FCA-4C92-A97E-BE065168CA42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -310,12 +310,18 @@
 assets/projects/wither app/Realme 10-3.png</t>
   </si>
   <si>
-    <t>assets/projects/marn/marn googleplay banner.png,
+    <t xml:space="preserve">assets/projects/marn/marn googleplay banner1.png,
 assets/projects/marn/remove bg.png,
-assets/projects/marn/5.png,
-assets/projects/marn/6.png,
-assets/projects/marn/7.png,
-assets/projects/marn/8.png</t>
+assets/projects/marn/Blue.svg,
+assets/projects/marn/Blue-1.svg,
+assets/projects/marn/Blue-2.svg,
+assets/projects/marn/Blue-3.svg,
+assets/projects/marn/Blue-4.svg,
+assets/projects/marn/Blue-5.svg,
+assets/projects/marn/Blue-6.svg,
+assets/projects/marn/Blue-7.svg,
+assets/projects/marn/Blue-8.svg
+</t>
   </si>
 </sst>
 </file>

</xml_diff>